<commit_message>
Se mejora validar ventas ml
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -4,17 +4,18 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="OMITIDOS" sheetId="1" r:id="rId1"/>
-    <sheet name="Stock ML" sheetId="2" r:id="rId2"/>
-    <sheet name="VARIANTES VALIDAR" sheetId="3" r:id="rId3"/>
+    <sheet name="Pack" sheetId="4" r:id="rId2"/>
+    <sheet name="Stock ML" sheetId="2" r:id="rId3"/>
+    <sheet name="VARIANTES VALIDAR" sheetId="3" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">OMITIDOS!$A$1:$A$38</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Stock ML'!$A$1:$B$31</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'VARIANTES VALIDAR'!$A$1:$A$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Stock ML'!$A$1:$B$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'VARIANTES VALIDAR'!$A$1:$A$54</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="134">
   <si>
     <t>Número Publicación</t>
   </si>
@@ -416,6 +417,18 @@
   </si>
   <si>
     <t>MLC1730850612</t>
+  </si>
+  <si>
+    <t>MLC938208013</t>
+  </si>
+  <si>
+    <t>MLC3341832018</t>
+  </si>
+  <si>
+    <t>MLC2889792602</t>
+  </si>
+  <si>
+    <t>MLC2889909014</t>
   </si>
 </sst>
 </file>
@@ -959,8 +972,8 @@
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A43" s="1">
-        <v>938208013</v>
+      <c r="A43" s="1" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.3">
@@ -1003,6 +1016,37 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="35" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>131</v>
+      </c>
+      <c r="B1" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:C32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1021,7 +1065,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -1029,7 +1073,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -1037,7 +1081,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -1045,7 +1089,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -1060,8 +1104,11 @@
       <c r="B6">
         <v>6</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -1069,7 +1116,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>20</v>
       </c>
@@ -1077,7 +1124,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>21</v>
       </c>
@@ -1085,7 +1132,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -1093,7 +1140,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>23</v>
       </c>
@@ -1104,7 +1151,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>24</v>
       </c>
@@ -1115,7 +1162,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>25</v>
       </c>
@@ -1126,7 +1173,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>26</v>
       </c>
@@ -1137,7 +1184,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>27</v>
       </c>
@@ -1145,7 +1192,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>28</v>
       </c>
@@ -1153,7 +1200,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>29</v>
       </c>
@@ -1161,7 +1208,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>30</v>
       </c>
@@ -1169,7 +1216,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>31</v>
       </c>
@@ -1177,7 +1224,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>32</v>
       </c>
@@ -1185,7 +1232,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>33</v>
       </c>
@@ -1196,7 +1243,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>34</v>
       </c>
@@ -1207,7 +1254,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>35</v>
       </c>
@@ -1215,7 +1262,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>36</v>
       </c>
@@ -1223,7 +1270,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>37</v>
       </c>
@@ -1231,7 +1278,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>38</v>
       </c>
@@ -1239,7 +1286,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>39</v>
       </c>
@@ -1247,7 +1294,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>40</v>
       </c>
@@ -1258,7 +1305,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>41</v>
       </c>
@@ -1266,7 +1313,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>42</v>
       </c>
@@ -1274,7 +1321,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>43</v>
       </c>
@@ -1282,7 +1329,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>32</v>
       </c>
@@ -1294,13 +1341,19 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B31"/>
+  <autoFilter ref="A1:B32">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="MLC1778567895"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="260" orientation="portrait" horizontalDpi="203" verticalDpi="203" r:id="rId1"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr filterMode="1"/>
   <dimension ref="A1:A54"/>

</xml_diff>

<commit_message>
Se integra pack a configuración
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="135">
   <si>
     <t>Número Publicación</t>
   </si>
@@ -429,6 +429,9 @@
   </si>
   <si>
     <t>MLC2889909014</t>
+  </si>
+  <si>
+    <t>MLC1772690125</t>
   </si>
 </sst>
 </file>
@@ -1016,7 +1019,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.6640625" bestFit="1" customWidth="1"/>
@@ -1039,8 +1042,25 @@
         <v>133</v>
       </c>
     </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B4" t="s">
+        <v>134</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="260" orientation="portrait" horizontalDpi="203" verticalDpi="203" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1097,7 +1117,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>18</v>
       </c>
@@ -1232,7 +1252,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="21" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>33</v>
       </c>
@@ -1344,7 +1364,7 @@
   <autoFilter ref="A1:B32">
     <filterColumn colId="0">
       <filters>
-        <filter val="MLC1778567895"/>
+        <filter val="MLC3394633770"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>

<commit_message>
Se integra compra internacional
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="OMITIDOS" sheetId="1" r:id="rId1"/>
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">OMITIDOS!$A$1:$A$38</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Stock ML'!$A$1:$B$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Stock ML'!$A$1:$B$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'VARIANTES VALIDAR'!$A$1:$A$54</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="135">
   <si>
     <t>Número Publicación</t>
   </si>
@@ -1047,7 +1047,7 @@
         <v>33</v>
       </c>
       <c r="B3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
@@ -1067,7 +1067,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.44140625" bestFit="1" customWidth="1"/>
@@ -1254,7 +1254,7 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B21">
         <v>6</v>
@@ -1265,18 +1265,15 @@
     </row>
     <row r="22" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B22">
         <v>6</v>
-      </c>
-      <c r="C22">
-        <v>3</v>
       </c>
     </row>
     <row r="23" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B23">
         <v>6</v>
@@ -1284,7 +1281,7 @@
     </row>
     <row r="24" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B24">
         <v>6</v>
@@ -1292,7 +1289,7 @@
     </row>
     <row r="25" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B25">
         <v>6</v>
@@ -1300,34 +1297,34 @@
     </row>
     <row r="26" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B26">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="27" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B27">
         <v>4</v>
       </c>
+      <c r="C27">
+        <v>2</v>
+      </c>
     </row>
     <row r="28" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B28">
         <v>4</v>
       </c>
-      <c r="C28">
-        <v>2</v>
-      </c>
     </row>
     <row r="29" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B29">
         <v>4</v>
@@ -1335,36 +1332,28 @@
     </row>
     <row r="30" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B30">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="31" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="B31">
         <v>6</v>
       </c>
-    </row>
-    <row r="32" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A32" t="s">
-        <v>32</v>
-      </c>
-      <c r="B32">
-        <v>6</v>
-      </c>
-      <c r="C32">
+      <c r="C31">
         <v>3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B32">
+  <autoFilter ref="A1:B31">
     <filterColumn colId="0">
       <filters>
-        <filter val="MLC3394633770"/>
+        <filter val="MLC3394910104"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>

<commit_message>
Se corrije lectura de paquetes validar-ml
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">OMITIDOS!$A$1:$A$38</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Pack!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Pack!$A$1:$B$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Stock ML'!$A$1:$B$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'VARIANTES VALIDAR'!$A$1:$A$54</definedName>
   </definedNames>
@@ -1065,6 +1065,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1080,7 +1081,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>131</v>
       </c>
@@ -1088,7 +1089,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>131</v>
       </c>
@@ -1096,7 +1097,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>135</v>
       </c>
@@ -1104,7 +1105,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>135</v>
       </c>
@@ -1112,7 +1113,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>135</v>
       </c>
@@ -1120,7 +1121,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>32</v>
       </c>
@@ -1128,7 +1129,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>32</v>
       </c>
@@ -1136,7 +1137,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>33</v>
       </c>
@@ -1144,7 +1145,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>33</v>
       </c>
@@ -1152,7 +1153,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>23</v>
       </c>
@@ -1160,7 +1161,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>23</v>
       </c>
@@ -1184,7 +1185,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>141</v>
       </c>
@@ -1192,7 +1193,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>141</v>
       </c>
@@ -1200,7 +1201,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>144</v>
       </c>
@@ -1208,7 +1209,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>144</v>
       </c>
@@ -1216,7 +1217,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>147</v>
       </c>
@@ -1224,7 +1225,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>147</v>
       </c>
@@ -1233,7 +1234,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B1"/>
+  <autoFilter ref="A1:B20">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="MLC3394633742"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="260" orientation="portrait" horizontalDpi="203" verticalDpi="203" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Se mejora carga de archivos desde carpeta y validadores
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -1065,7 +1065,6 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1081,7 +1080,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="2" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>131</v>
       </c>
@@ -1089,7 +1088,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="3" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>131</v>
       </c>
@@ -1097,7 +1096,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="4" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>135</v>
       </c>
@@ -1105,7 +1104,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="5" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>135</v>
       </c>
@@ -1113,7 +1112,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="6" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>135</v>
       </c>
@@ -1121,7 +1120,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="7" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>32</v>
       </c>
@@ -1129,7 +1128,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="8" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>32</v>
       </c>
@@ -1137,7 +1136,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>33</v>
       </c>
@@ -1145,7 +1144,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="10" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>33</v>
       </c>
@@ -1153,7 +1152,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="11" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>23</v>
       </c>
@@ -1161,7 +1160,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>23</v>
       </c>
@@ -1185,7 +1184,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="15" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>141</v>
       </c>
@@ -1193,7 +1192,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="16" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>141</v>
       </c>
@@ -1201,7 +1200,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="17" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>144</v>
       </c>
@@ -1209,7 +1208,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="18" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>144</v>
       </c>
@@ -1217,7 +1216,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="19" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>147</v>
       </c>
@@ -1225,7 +1224,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="20" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>147</v>
       </c>
@@ -1234,13 +1233,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B20">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="MLC3394633742"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:B20"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="260" orientation="portrait" horizontalDpi="203" verticalDpi="203" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Se integran publicaciones adicionales a compra internacional
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="OMITIDOS" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="155">
   <si>
     <t>Número Publicación</t>
   </si>
@@ -478,6 +478,21 @@
   </si>
   <si>
     <t>MLC636399648</t>
+  </si>
+  <si>
+    <t>MLC1033139189</t>
+  </si>
+  <si>
+    <t>MLC1313890468</t>
+  </si>
+  <si>
+    <t>MLC1313823753</t>
+  </si>
+  <si>
+    <t>MLC1292021203</t>
+  </si>
+  <si>
+    <t>MLC1383929703</t>
   </si>
 </sst>
 </file>
@@ -1065,7 +1080,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.6640625" bestFit="1" customWidth="1"/>
@@ -1230,6 +1245,38 @@
       </c>
       <c r="B20" t="s">
         <v>149</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>153</v>
+      </c>
+      <c r="B21" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>153</v>
+      </c>
+      <c r="B22" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>150</v>
+      </c>
+      <c r="B23" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>150</v>
+      </c>
+      <c r="B24" t="s">
+        <v>152</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Se mejora integra escaneo modo supervisor
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="OMITIDOS" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="156">
   <si>
     <t>Número Publicación</t>
   </si>
@@ -493,6 +493,9 @@
   </si>
   <si>
     <t>MLC1383929703</t>
+  </si>
+  <si>
+    <t>MLC1900551185</t>
   </si>
 </sst>
 </file>
@@ -1288,8 +1291,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.44140625" bestFit="1" customWidth="1"/>
@@ -1307,7 +1309,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="2" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -1315,7 +1317,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -1323,7 +1325,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -1331,7 +1333,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -1339,7 +1341,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>18</v>
       </c>
@@ -1350,7 +1352,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -1358,7 +1360,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>20</v>
       </c>
@@ -1366,7 +1368,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>21</v>
       </c>
@@ -1374,7 +1376,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -1382,7 +1384,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>23</v>
       </c>
@@ -1393,7 +1395,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>24</v>
       </c>
@@ -1404,7 +1406,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>25</v>
       </c>
@@ -1415,7 +1417,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>26</v>
       </c>
@@ -1426,7 +1428,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>27</v>
       </c>
@@ -1434,7 +1436,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="16" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>28</v>
       </c>
@@ -1442,7 +1444,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="17" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>29</v>
       </c>
@@ -1450,7 +1452,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="18" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>30</v>
       </c>
@@ -1458,7 +1460,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="19" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>31</v>
       </c>
@@ -1466,7 +1468,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="20" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>32</v>
       </c>
@@ -1474,7 +1476,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="21" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>34</v>
       </c>
@@ -1485,7 +1487,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>35</v>
       </c>
@@ -1493,7 +1495,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="23" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>36</v>
       </c>
@@ -1501,7 +1503,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="24" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>37</v>
       </c>
@@ -1509,7 +1511,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="25" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>38</v>
       </c>
@@ -1517,7 +1519,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="26" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>39</v>
       </c>
@@ -1536,7 +1538,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="28" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>41</v>
       </c>
@@ -1544,7 +1546,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="29" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>42</v>
       </c>
@@ -1552,7 +1554,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="30" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>43</v>
       </c>
@@ -1560,7 +1562,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="31" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>32</v>
       </c>
@@ -1571,14 +1573,16 @@
         <v>3</v>
       </c>
     </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>155</v>
+      </c>
+      <c r="B32">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B31">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="MLC1629789897"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:B31"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="260" orientation="portrait" horizontalDpi="203" verticalDpi="203" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Se configura paquete reposapiés CB190R Originales
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="OMITIDOS" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="159">
   <si>
     <t>Número Publicación</t>
   </si>
@@ -496,6 +496,15 @@
   </si>
   <si>
     <t>MLC1900551185</t>
+  </si>
+  <si>
+    <t>MLC2013914492</t>
+  </si>
+  <si>
+    <t>MLC2554626296</t>
+  </si>
+  <si>
+    <t>MLC1500535503</t>
   </si>
 </sst>
 </file>
@@ -1083,7 +1092,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.6640625" bestFit="1" customWidth="1"/>
@@ -1280,6 +1289,22 @@
       </c>
       <c r="B24" t="s">
         <v>152</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>156</v>
+      </c>
+      <c r="B25" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>156</v>
+      </c>
+      <c r="B26" t="s">
+        <v>158</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Se arregla precio venta-jumpseller despacho Santiago
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="161">
   <si>
     <t>Número Publicación</t>
   </si>
@@ -505,6 +505,12 @@
   </si>
   <si>
     <t>MLC1500535503</t>
+  </si>
+  <si>
+    <t>MLC3851485578</t>
+  </si>
+  <si>
+    <t>MLC1916418509</t>
   </si>
 </sst>
 </file>
@@ -1316,7 +1322,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C34"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.44140625" bestFit="1" customWidth="1"/>
@@ -1604,6 +1610,22 @@
       </c>
       <c r="B32">
         <v>6</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>159</v>
+      </c>
+      <c r="B33">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>160</v>
+      </c>
+      <c r="B34">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Se configura pack aceites yamalube
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" firstSheet="1" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="OMITIDOS" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="163">
   <si>
     <t>Número Publicación</t>
   </si>
@@ -511,6 +511,12 @@
   </si>
   <si>
     <t>MLC1916418509</t>
+  </si>
+  <si>
+    <t>MLC1914208353</t>
+  </si>
+  <si>
+    <t>MLC3872436310</t>
   </si>
 </sst>
 </file>
@@ -1098,7 +1104,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.6640625" bestFit="1" customWidth="1"/>
@@ -1313,6 +1319,22 @@
         <v>158</v>
       </c>
     </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>161</v>
+      </c>
+      <c r="B27" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>161</v>
+      </c>
+      <c r="B28" t="s">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:B20"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1322,7 +1344,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.44140625" bestFit="1" customWidth="1"/>
@@ -1612,7 +1634,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>159</v>
       </c>
@@ -1620,12 +1642,23 @@
         <v>14</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>160</v>
       </c>
       <c r="B34">
         <v>12</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>162</v>
+      </c>
+      <c r="B35">
+        <v>6</v>
+      </c>
+      <c r="C35">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Se corrige configuración de packs
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="168">
   <si>
     <t>Número Publicación</t>
   </si>
@@ -517,6 +517,21 @@
   </si>
   <si>
     <t>MLC3872436310</t>
+  </si>
+  <si>
+    <t>MLC1320686626</t>
+  </si>
+  <si>
+    <t>MLC1931459349</t>
+  </si>
+  <si>
+    <t>MLC2865524730</t>
+  </si>
+  <si>
+    <t>MLC1931501759</t>
+  </si>
+  <si>
+    <t>MLC1931540207</t>
   </si>
 </sst>
 </file>
@@ -1104,7 +1119,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B28"/>
+  <dimension ref="A1:B32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.6640625" bestFit="1" customWidth="1"/>
@@ -1333,6 +1348,38 @@
       </c>
       <c r="B28" t="s">
         <v>15</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>163</v>
+      </c>
+      <c r="B29" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>163</v>
+      </c>
+      <c r="B30" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>163</v>
+      </c>
+      <c r="B31" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>163</v>
+      </c>
+      <c r="B32" t="s">
+        <v>167</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Se configura pack yamalube + filtro aceite fz25
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" firstSheet="1" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="OMITIDOS" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="172">
   <si>
     <t>Número Publicación</t>
   </si>
@@ -532,6 +532,18 @@
   </si>
   <si>
     <t>MLC1931540207</t>
+  </si>
+  <si>
+    <t>MLC967212574</t>
+  </si>
+  <si>
+    <t>MLC3841877700</t>
+  </si>
+  <si>
+    <t>MLC3907665240</t>
+  </si>
+  <si>
+    <t>MLC1658524699</t>
   </si>
 </sst>
 </file>
@@ -858,7 +870,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:A48"/>
+  <dimension ref="A1:A49"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.44140625" style="1" bestFit="1" customWidth="1"/>
@@ -1102,6 +1114,11 @@
     <row r="48" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
         <v>129</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A49" s="1" t="s">
+        <v>168</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1136,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B32"/>
+  <dimension ref="A1:B34"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.6640625" bestFit="1" customWidth="1"/>
@@ -1382,6 +1399,22 @@
         <v>167</v>
       </c>
     </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>169</v>
+      </c>
+      <c r="B33" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>169</v>
+      </c>
+      <c r="B34" t="s">
+        <v>171</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:B20"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1391,7 +1424,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.44140625" bestFit="1" customWidth="1"/>
@@ -1706,6 +1739,17 @@
       </c>
       <c r="C35">
         <v>3</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>170</v>
+      </c>
+      <c r="B36">
+        <v>4</v>
+      </c>
+      <c r="C36">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Se integra validación de no entregadas para ventas canceladas y confirmar despacho de cantidades > 2 en jumpseller
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -14,8 +14,8 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">OMITIDOS!$A$1:$A$38</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Pack!$A$1:$B$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Stock ML'!$A$1:$B$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Pack!$A$1:$B$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Stock ML'!$A$1:$B$38</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'VARIANTES VALIDAR'!$A$1:$A$54</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="173">
   <si>
     <t>Número Publicación</t>
   </si>
@@ -544,6 +544,9 @@
   </si>
   <si>
     <t>MLC1658524699</t>
+  </si>
+  <si>
+    <t>MLC1774163439</t>
   </si>
 </sst>
 </file>
@@ -1416,7 +1419,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B20"/>
+  <autoFilter ref="A1:B34"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="260" orientation="portrait" horizontalDpi="203" verticalDpi="203" r:id="rId1"/>
 </worksheet>
@@ -1424,7 +1427,8 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C36"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:C38"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.44140625" bestFit="1" customWidth="1"/>
@@ -1442,7 +1446,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -1450,7 +1454,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -1458,7 +1462,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -1466,7 +1470,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -1479,13 +1483,13 @@
         <v>18</v>
       </c>
       <c r="B6">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C6">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -1493,7 +1497,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>20</v>
       </c>
@@ -1501,7 +1505,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>21</v>
       </c>
@@ -1509,7 +1513,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -1517,7 +1521,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>23</v>
       </c>
@@ -1528,7 +1532,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>24</v>
       </c>
@@ -1539,7 +1543,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>25</v>
       </c>
@@ -1550,7 +1554,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>26</v>
       </c>
@@ -1561,7 +1565,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>27</v>
       </c>
@@ -1569,7 +1573,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>28</v>
       </c>
@@ -1577,7 +1581,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>29</v>
       </c>
@@ -1585,7 +1589,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>30</v>
       </c>
@@ -1593,7 +1597,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>31</v>
       </c>
@@ -1601,7 +1605,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>32</v>
       </c>
@@ -1609,7 +1613,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>34</v>
       </c>
@@ -1620,7 +1624,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>35</v>
       </c>
@@ -1628,7 +1632,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>36</v>
       </c>
@@ -1636,7 +1640,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>37</v>
       </c>
@@ -1644,7 +1648,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>38</v>
       </c>
@@ -1652,7 +1656,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>39</v>
       </c>
@@ -1660,7 +1664,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>40</v>
       </c>
@@ -1671,7 +1675,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>41</v>
       </c>
@@ -1679,7 +1683,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>42</v>
       </c>
@@ -1687,7 +1691,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>43</v>
       </c>
@@ -1695,7 +1699,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>32</v>
       </c>
@@ -1706,15 +1710,15 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>155</v>
       </c>
       <c r="B32">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>159</v>
       </c>
@@ -1722,7 +1726,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>160</v>
       </c>
@@ -1730,7 +1734,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>162</v>
       </c>
@@ -1741,19 +1745,41 @@
         <v>3</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>170</v>
       </c>
       <c r="B36">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C36">
         <v>2</v>
       </c>
     </row>
+    <row r="37" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>171</v>
+      </c>
+      <c r="B37">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>172</v>
+      </c>
+      <c r="B38">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B31"/>
+  <autoFilter ref="A1:B38">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="MLC1778567895"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="260" orientation="portrait" horizontalDpi="203" verticalDpi="203" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Se corrige búsqueda de códigos ventas particulares en referencia interna para match
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">OMITIDOS!$A$1:$A$38</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Pack!$A$1:$B$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Stock ML'!$A$1:$B$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Stock ML'!$A$1:$B$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'VARIANTES VALIDAR'!$A$1:$A$54</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="174">
   <si>
     <t>Número Publicación</t>
   </si>
@@ -547,6 +547,9 @@
   </si>
   <si>
     <t>MLC1774163439</t>
+  </si>
+  <si>
+    <t>MLC3940038744</t>
   </si>
 </sst>
 </file>
@@ -1428,7 +1431,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.44140625" bestFit="1" customWidth="1"/>
@@ -1478,7 +1481,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>18</v>
       </c>
@@ -1772,11 +1775,19 @@
         <v>6</v>
       </c>
     </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>173</v>
+      </c>
+      <c r="B39">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B38">
+  <autoFilter ref="A1:B39">
     <filterColumn colId="0">
       <filters>
-        <filter val="MLC1778567895"/>
+        <filter val="MLC3940038744"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>

<commit_message>
Se actualiza configuración pack
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="176">
   <si>
     <t>Número Publicación</t>
   </si>
@@ -550,6 +550,12 @@
   </si>
   <si>
     <t>MLC3940038744</t>
+  </si>
+  <si>
+    <t>MLC3968074452</t>
+  </si>
+  <si>
+    <t>MLC3965075300</t>
   </si>
 </sst>
 </file>
@@ -1430,8 +1436,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.44140625" bestFit="1" customWidth="1"/>
@@ -1449,7 +1454,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="2" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -1457,7 +1462,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -1465,7 +1470,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -1473,7 +1478,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -1481,7 +1486,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>18</v>
       </c>
@@ -1492,7 +1497,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -1500,7 +1505,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>20</v>
       </c>
@@ -1508,7 +1513,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>21</v>
       </c>
@@ -1516,7 +1521,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -1524,7 +1529,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>23</v>
       </c>
@@ -1535,7 +1540,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>24</v>
       </c>
@@ -1546,7 +1551,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>25</v>
       </c>
@@ -1557,7 +1562,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>26</v>
       </c>
@@ -1568,7 +1573,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>27</v>
       </c>
@@ -1576,7 +1581,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="16" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>28</v>
       </c>
@@ -1584,7 +1589,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="17" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>29</v>
       </c>
@@ -1592,7 +1597,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="18" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>30</v>
       </c>
@@ -1600,7 +1605,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="19" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>31</v>
       </c>
@@ -1608,7 +1613,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="20" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>32</v>
       </c>
@@ -1616,7 +1621,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="21" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>34</v>
       </c>
@@ -1627,7 +1632,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>35</v>
       </c>
@@ -1635,7 +1640,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="23" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>36</v>
       </c>
@@ -1643,7 +1648,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="24" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>37</v>
       </c>
@@ -1651,7 +1656,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="25" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>38</v>
       </c>
@@ -1659,7 +1664,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="26" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>39</v>
       </c>
@@ -1667,7 +1672,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="27" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>40</v>
       </c>
@@ -1678,7 +1683,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="28" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>41</v>
       </c>
@@ -1686,7 +1691,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="29" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>42</v>
       </c>
@@ -1694,7 +1699,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="30" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>43</v>
       </c>
@@ -1702,7 +1707,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="31" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>32</v>
       </c>
@@ -1713,7 +1718,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>155</v>
       </c>
@@ -1721,7 +1726,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="33" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>159</v>
       </c>
@@ -1729,7 +1734,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="34" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>160</v>
       </c>
@@ -1737,7 +1742,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="35" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>162</v>
       </c>
@@ -1748,7 +1753,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="36" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>170</v>
       </c>
@@ -1759,7 +1764,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>171</v>
       </c>
@@ -1767,7 +1772,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="38" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>172</v>
       </c>
@@ -1783,14 +1788,24 @@
         <v>6</v>
       </c>
     </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>174</v>
+      </c>
+      <c r="B40">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>175</v>
+      </c>
+      <c r="B41">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B39">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="MLC3940038744"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:B39"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="260" orientation="portrait" horizontalDpi="203" verticalDpi="203" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Se actualiza configuración pack 2
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="177">
   <si>
     <t>Número Publicación</t>
   </si>
@@ -556,6 +556,9 @@
   </si>
   <si>
     <t>MLC3965075300</t>
+  </si>
+  <si>
+    <t>MLC1972672845</t>
   </si>
 </sst>
 </file>
@@ -1436,7 +1439,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:C42"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.44140625" bestFit="1" customWidth="1"/>
@@ -1802,6 +1805,14 @@
       </c>
       <c r="B41">
         <v>6</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>176</v>
+      </c>
+      <c r="B42">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Se actualiza configuración pack 3
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="178">
   <si>
     <t>Número Publicación</t>
   </si>
@@ -559,6 +559,9 @@
   </si>
   <si>
     <t>MLC1972672845</t>
+  </si>
+  <si>
+    <t>MLC3922959212</t>
   </si>
 </sst>
 </file>
@@ -1439,7 +1442,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C43"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.44140625" bestFit="1" customWidth="1"/>
@@ -1813,6 +1816,14 @@
       </c>
       <c r="B42">
         <v>8</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>177</v>
+      </c>
+      <c r="B43">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Se configura filtro aceite con 4 unidades
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="OMITIDOS" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="178">
   <si>
     <t>Número Publicación</t>
   </si>
@@ -1442,7 +1442,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C43"/>
+  <dimension ref="A1:C44"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.44140625" bestFit="1" customWidth="1"/>
@@ -1823,6 +1823,14 @@
         <v>177</v>
       </c>
       <c r="B43">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>15</v>
+      </c>
+      <c r="B44">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Se actualiza configuración publicaciones
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="180">
   <si>
     <t>Número Publicación</t>
   </si>
@@ -562,6 +562,12 @@
   </si>
   <si>
     <t>MLC3922959212</t>
+  </si>
+  <si>
+    <t>MLC1949786775</t>
+  </si>
+  <si>
+    <t>MLC1949799733</t>
   </si>
 </sst>
 </file>
@@ -1442,7 +1448,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C44"/>
+  <dimension ref="A1:C46"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.44140625" bestFit="1" customWidth="1"/>
@@ -1832,6 +1838,28 @@
       </c>
       <c r="B44">
         <v>4</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>178</v>
+      </c>
+      <c r="B45">
+        <v>14</v>
+      </c>
+      <c r="C45">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>179</v>
+      </c>
+      <c r="B46">
+        <v>12</v>
+      </c>
+      <c r="C46">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Se modifica lógica para trabajar con opciones
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="OMITIDOS" sheetId="1" r:id="rId1"/>
@@ -13,7 +13,7 @@
     <sheet name="VARIANTES VALIDAR" sheetId="3" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">OMITIDOS!$A$1:$A$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">OMITIDOS!$A$1:$A$49</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Pack!$A$1:$B$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Stock ML'!$A$1:$B$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'VARIANTES VALIDAR'!$A$1:$A$54</definedName>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="181">
   <si>
     <t>Número Publicación</t>
   </si>
@@ -568,6 +568,9 @@
   </si>
   <si>
     <t>MLC1949799733</t>
+  </si>
+  <si>
+    <t>OP1</t>
   </si>
 </sst>
 </file>
@@ -893,7 +896,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:A49"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -905,182 +907,182 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>1589202743</v>
       </c>
     </row>
-    <row r="5" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="16" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="17" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="18" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="19" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="20" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="21" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="22" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="23" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="24" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="25" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="26" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="27" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="28" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="29" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="30" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="31" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="32" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="33" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" s="1">
         <v>973038687</v>
       </c>
     </row>
-    <row r="34" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="35" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="36" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="37" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
         <v>119</v>
       </c>
@@ -1146,13 +1148,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:A38">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="MLC1589202743"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:A49"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="260" orientation="portrait" horizontalDpi="203" verticalDpi="203" r:id="rId1"/>
 </worksheet>
@@ -1160,14 +1156,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B34"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:C34"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="35" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>140</v>
       </c>
@@ -1175,7 +1172,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>131</v>
       </c>
@@ -1183,7 +1180,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>131</v>
       </c>
@@ -1191,23 +1188,29 @@
         <v>133</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>135</v>
       </c>
       <c r="B4" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C4" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>135</v>
       </c>
       <c r="B5" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C5" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>135</v>
       </c>
@@ -1215,7 +1218,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>32</v>
       </c>
@@ -1223,7 +1226,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>32</v>
       </c>
@@ -1231,7 +1234,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>33</v>
       </c>
@@ -1239,7 +1242,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>33</v>
       </c>
@@ -1247,7 +1250,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>23</v>
       </c>
@@ -1255,7 +1258,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>23</v>
       </c>
@@ -1263,7 +1266,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>24</v>
       </c>
@@ -1271,7 +1274,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>24</v>
       </c>
@@ -1279,7 +1282,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>141</v>
       </c>
@@ -1287,7 +1290,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>141</v>
       </c>
@@ -1295,7 +1298,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>144</v>
       </c>
@@ -1303,7 +1306,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>144</v>
       </c>
@@ -1311,7 +1314,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>147</v>
       </c>
@@ -1319,7 +1322,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>147</v>
       </c>
@@ -1327,7 +1330,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>153</v>
       </c>
@@ -1335,7 +1338,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>153</v>
       </c>
@@ -1343,7 +1346,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>150</v>
       </c>
@@ -1351,7 +1354,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>150</v>
       </c>
@@ -1359,7 +1362,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>156</v>
       </c>
@@ -1367,7 +1370,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>156</v>
       </c>
@@ -1375,7 +1378,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>161</v>
       </c>
@@ -1383,7 +1386,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>161</v>
       </c>
@@ -1391,7 +1394,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>163</v>
       </c>
@@ -1399,7 +1402,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>163</v>
       </c>
@@ -1407,7 +1410,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>163</v>
       </c>
@@ -1415,7 +1418,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>163</v>
       </c>
@@ -1423,7 +1426,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>169</v>
       </c>
@@ -1431,7 +1434,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>169</v>
       </c>
@@ -1440,7 +1443,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B34"/>
+  <autoFilter ref="A1:B34">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="MLC1143851763"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="260" orientation="portrait" horizontalDpi="203" verticalDpi="203" r:id="rId1"/>
 </worksheet>
@@ -1871,7 +1880,6 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:A54"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1883,82 +1891,82 @@
         <v>62</v>
       </c>
     </row>
-    <row r="2" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="3" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="5" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="6" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="7" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="8" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="9" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="10" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="11" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="12" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="13" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="14" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="15" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="16" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="17" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>78</v>
       </c>
@@ -1968,194 +1976,188 @@
         <v>79</v>
       </c>
     </row>
-    <row r="19" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="20" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="21" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="22" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="23" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="24" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="25" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="26" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="27" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="28" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="29" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="30" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="31" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="32" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="33" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="34" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="35" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="36" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="37" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="38" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="39" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="40" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="41" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="42" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="43" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="44" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="45" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="46" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="47" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="48" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="49" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="50" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="51" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="52" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="53" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="54" spans="1:1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>115</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:A54">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="Rojo-Negro-Rojo"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:A54"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Se modifica configuración kit mantención yamalube
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">OMITIDOS!$A$1:$A$49</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Pack!$A$1:$B$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Stock ML'!$A$1:$B$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Stock ML'!$A$1:$B$46</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'VARIANTES VALIDAR'!$A$1:$A$54</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="185">
   <si>
     <t>Número Publicación</t>
   </si>
@@ -571,6 +571,18 @@
   </si>
   <si>
     <t>OP1</t>
+  </si>
+  <si>
+    <t>MLC2061579003</t>
+  </si>
+  <si>
+    <t>MLC2018304139</t>
+  </si>
+  <si>
+    <t>MLC2018355097</t>
+  </si>
+  <si>
+    <t>MLC2018355127</t>
   </si>
 </sst>
 </file>
@@ -1156,8 +1168,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C40"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.6640625" bestFit="1" customWidth="1"/>
@@ -1172,7 +1183,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>131</v>
       </c>
@@ -1180,7 +1191,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>131</v>
       </c>
@@ -1218,7 +1229,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>32</v>
       </c>
@@ -1226,7 +1237,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>32</v>
       </c>
@@ -1234,7 +1245,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>33</v>
       </c>
@@ -1242,7 +1253,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>33</v>
       </c>
@@ -1250,7 +1261,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>23</v>
       </c>
@@ -1258,7 +1269,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>23</v>
       </c>
@@ -1266,7 +1277,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>24</v>
       </c>
@@ -1274,7 +1285,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>24</v>
       </c>
@@ -1282,7 +1293,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>141</v>
       </c>
@@ -1290,7 +1301,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>141</v>
       </c>
@@ -1298,7 +1309,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>144</v>
       </c>
@@ -1306,7 +1317,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>144</v>
       </c>
@@ -1314,7 +1325,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>147</v>
       </c>
@@ -1322,7 +1333,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>147</v>
       </c>
@@ -1330,7 +1341,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>153</v>
       </c>
@@ -1338,7 +1349,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>153</v>
       </c>
@@ -1346,7 +1357,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>150</v>
       </c>
@@ -1354,7 +1365,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>150</v>
       </c>
@@ -1362,7 +1373,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>156</v>
       </c>
@@ -1370,7 +1381,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>156</v>
       </c>
@@ -1378,7 +1389,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="27" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>161</v>
       </c>
@@ -1386,7 +1397,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="28" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>161</v>
       </c>
@@ -1394,7 +1405,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="29" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>163</v>
       </c>
@@ -1402,7 +1413,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="30" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>163</v>
       </c>
@@ -1410,7 +1421,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="31" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>163</v>
       </c>
@@ -1418,7 +1429,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="32" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>163</v>
       </c>
@@ -1426,7 +1437,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="33" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>169</v>
       </c>
@@ -1434,7 +1445,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="34" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>169</v>
       </c>
@@ -1442,13 +1453,59 @@
         <v>171</v>
       </c>
     </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>182</v>
+      </c>
+      <c r="B35" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>182</v>
+      </c>
+      <c r="B36" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>183</v>
+      </c>
+      <c r="B37" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>183</v>
+      </c>
+      <c r="B38" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>184</v>
+      </c>
+      <c r="B39" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>184</v>
+      </c>
+      <c r="B40" t="s">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:B34">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="MLC1143851763"/>
-      </filters>
-    </filterColumn>
+    <sortState ref="A4:B6">
+      <sortCondition descending="1" ref="A1:A34"/>
+    </sortState>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="260" orientation="portrait" horizontalDpi="203" verticalDpi="203" r:id="rId1"/>
@@ -1457,7 +1514,8 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C46"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:C47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.44140625" bestFit="1" customWidth="1"/>
@@ -1475,7 +1533,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -1483,7 +1541,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -1491,7 +1549,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -1499,7 +1557,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -1507,7 +1565,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>18</v>
       </c>
@@ -1518,7 +1576,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -1526,7 +1584,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>20</v>
       </c>
@@ -1534,7 +1592,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>21</v>
       </c>
@@ -1542,7 +1600,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -1550,7 +1608,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>23</v>
       </c>
@@ -1561,7 +1619,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>24</v>
       </c>
@@ -1572,7 +1630,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>25</v>
       </c>
@@ -1583,7 +1641,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>26</v>
       </c>
@@ -1594,7 +1652,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>27</v>
       </c>
@@ -1602,7 +1660,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>28</v>
       </c>
@@ -1610,7 +1668,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>29</v>
       </c>
@@ -1618,7 +1676,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>30</v>
       </c>
@@ -1626,7 +1684,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>31</v>
       </c>
@@ -1634,7 +1692,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>32</v>
       </c>
@@ -1642,7 +1700,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>34</v>
       </c>
@@ -1653,7 +1711,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>35</v>
       </c>
@@ -1661,7 +1719,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>36</v>
       </c>
@@ -1669,7 +1727,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>37</v>
       </c>
@@ -1677,7 +1735,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>38</v>
       </c>
@@ -1685,7 +1743,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>39</v>
       </c>
@@ -1693,7 +1751,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>40</v>
       </c>
@@ -1704,7 +1762,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>41</v>
       </c>
@@ -1712,7 +1770,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>42</v>
       </c>
@@ -1720,7 +1778,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>43</v>
       </c>
@@ -1728,7 +1786,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>32</v>
       </c>
@@ -1739,7 +1797,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>155</v>
       </c>
@@ -1747,7 +1805,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>159</v>
       </c>
@@ -1755,7 +1813,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>160</v>
       </c>
@@ -1774,7 +1832,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>170</v>
       </c>
@@ -1785,7 +1843,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>171</v>
       </c>
@@ -1793,7 +1851,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>172</v>
       </c>
@@ -1801,7 +1859,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>173</v>
       </c>
@@ -1809,7 +1867,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>174</v>
       </c>
@@ -1817,7 +1875,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>175</v>
       </c>
@@ -1825,7 +1883,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>176</v>
       </c>
@@ -1833,7 +1891,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>177</v>
       </c>
@@ -1841,7 +1899,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>15</v>
       </c>
@@ -1849,7 +1907,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>178</v>
       </c>
@@ -1860,7 +1918,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>179</v>
       </c>
@@ -1871,8 +1929,25 @@
         <v>6</v>
       </c>
     </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>181</v>
+      </c>
+      <c r="B47">
+        <v>8</v>
+      </c>
+      <c r="C47">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B39"/>
+  <autoFilter ref="A1:B46">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="MLC3872436310"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="260" orientation="portrait" horizontalDpi="203" verticalDpi="203" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Se integra Reclamo cerrado con reembolso al comprador como cancelado
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="OMITIDOS" sheetId="1" r:id="rId1"/>
@@ -14,8 +14,8 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">OMITIDOS!$A$1:$A$49</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Pack!$A$1:$B$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Stock ML'!$A$1:$B$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Pack!$A$1:$B$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Stock ML'!$A$1:$B$47</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'VARIANTES VALIDAR'!$A$1:$A$54</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
@@ -1168,6 +1168,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:C40"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1183,7 +1184,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>131</v>
       </c>
@@ -1191,7 +1192,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>131</v>
       </c>
@@ -1199,7 +1200,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>135</v>
       </c>
@@ -1210,7 +1211,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>135</v>
       </c>
@@ -1221,7 +1222,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>135</v>
       </c>
@@ -1229,7 +1230,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>32</v>
       </c>
@@ -1237,7 +1238,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>32</v>
       </c>
@@ -1245,7 +1246,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>33</v>
       </c>
@@ -1253,7 +1254,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>33</v>
       </c>
@@ -1261,7 +1262,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>23</v>
       </c>
@@ -1269,7 +1270,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>23</v>
       </c>
@@ -1277,7 +1278,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>24</v>
       </c>
@@ -1285,7 +1286,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>24</v>
       </c>
@@ -1293,7 +1294,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>141</v>
       </c>
@@ -1301,7 +1302,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>141</v>
       </c>
@@ -1309,7 +1310,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>144</v>
       </c>
@@ -1317,7 +1318,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>144</v>
       </c>
@@ -1325,7 +1326,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>147</v>
       </c>
@@ -1333,7 +1334,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>147</v>
       </c>
@@ -1341,7 +1342,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>153</v>
       </c>
@@ -1349,7 +1350,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>153</v>
       </c>
@@ -1357,7 +1358,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>150</v>
       </c>
@@ -1365,7 +1366,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>150</v>
       </c>
@@ -1373,7 +1374,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>156</v>
       </c>
@@ -1381,7 +1382,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>156</v>
       </c>
@@ -1389,7 +1390,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="27" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>161</v>
       </c>
@@ -1397,7 +1398,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="28" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>161</v>
       </c>
@@ -1405,7 +1406,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="29" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>163</v>
       </c>
@@ -1413,7 +1414,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="30" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>163</v>
       </c>
@@ -1421,7 +1422,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="31" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>163</v>
       </c>
@@ -1429,7 +1430,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="32" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>163</v>
       </c>
@@ -1437,7 +1438,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="33" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>169</v>
       </c>
@@ -1445,7 +1446,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="34" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>169</v>
       </c>
@@ -1461,7 +1462,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>182</v>
       </c>
@@ -1477,7 +1478,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>183</v>
       </c>
@@ -1493,7 +1494,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>184</v>
       </c>
@@ -1502,7 +1503,12 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B34">
+  <autoFilter ref="A1:B40">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="MLC2061579003"/>
+      </filters>
+    </filterColumn>
     <sortState ref="A4:B6">
       <sortCondition descending="1" ref="A1:A34"/>
     </sortState>
@@ -1821,7 +1827,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>162</v>
       </c>
@@ -1941,10 +1947,10 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B46">
+  <autoFilter ref="A1:B47">
     <filterColumn colId="0">
       <filters>
-        <filter val="MLC3872436310"/>
+        <filter val="MLC2061579003"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>

<commit_message>
Se configura kit xmax 300
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="OMITIDOS" sheetId="1" r:id="rId1"/>
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">OMITIDOS!$A$1:$A$49</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Pack!$A$1:$B$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Pack!$A$1:$B$42</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Stock ML'!$A$1:$B$47</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'VARIANTES VALIDAR'!$A$1:$A$54</definedName>
   </definedNames>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="186">
   <si>
     <t>Número Publicación</t>
   </si>
@@ -583,6 +583,9 @@
   </si>
   <si>
     <t>MLC2018355127</t>
+  </si>
+  <si>
+    <t>MLC4105697882</t>
   </si>
 </sst>
 </file>
@@ -1169,7 +1172,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:C42"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.6640625" bestFit="1" customWidth="1"/>
@@ -1454,7 +1457,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>182</v>
       </c>
@@ -1470,7 +1473,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>183</v>
       </c>
@@ -1494,7 +1497,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="40" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>184</v>
       </c>
@@ -1502,11 +1505,27 @@
         <v>15</v>
       </c>
     </row>
+    <row r="41" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>185</v>
+      </c>
+      <c r="B41" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>185</v>
+      </c>
+      <c r="B42" t="s">
+        <v>171</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B40">
-    <filterColumn colId="1">
+  <autoFilter ref="A1:B42">
+    <filterColumn colId="0">
       <filters>
-        <filter val="MLC2061579003"/>
+        <filter val="MLC2018355127"/>
       </filters>
     </filterColumn>
     <sortState ref="A4:B6">
@@ -1520,7 +1539,6 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:C47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1539,7 +1557,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="2" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -1547,7 +1565,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -1555,7 +1573,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -1563,7 +1581,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -1571,7 +1589,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>18</v>
       </c>
@@ -1582,7 +1600,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -1590,7 +1608,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>20</v>
       </c>
@@ -1598,7 +1616,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>21</v>
       </c>
@@ -1606,7 +1624,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -1614,7 +1632,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>23</v>
       </c>
@@ -1625,7 +1643,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>24</v>
       </c>
@@ -1636,7 +1654,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>25</v>
       </c>
@@ -1647,7 +1665,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>26</v>
       </c>
@@ -1658,7 +1676,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>27</v>
       </c>
@@ -1666,7 +1684,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="16" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>28</v>
       </c>
@@ -1674,7 +1692,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="17" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>29</v>
       </c>
@@ -1682,7 +1700,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="18" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>30</v>
       </c>
@@ -1690,7 +1708,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="19" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>31</v>
       </c>
@@ -1698,7 +1716,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="20" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>32</v>
       </c>
@@ -1706,7 +1724,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="21" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>34</v>
       </c>
@@ -1717,7 +1735,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>35</v>
       </c>
@@ -1725,7 +1743,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="23" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>36</v>
       </c>
@@ -1733,7 +1751,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="24" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>37</v>
       </c>
@@ -1741,7 +1759,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="25" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>38</v>
       </c>
@@ -1749,7 +1767,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="26" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>39</v>
       </c>
@@ -1757,7 +1775,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="27" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>40</v>
       </c>
@@ -1768,7 +1786,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="28" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>41</v>
       </c>
@@ -1776,7 +1794,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="29" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>42</v>
       </c>
@@ -1784,7 +1802,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="30" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>43</v>
       </c>
@@ -1792,7 +1810,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="31" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>32</v>
       </c>
@@ -1803,7 +1821,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>155</v>
       </c>
@@ -1811,7 +1829,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="33" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>159</v>
       </c>
@@ -1819,7 +1837,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="34" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>160</v>
       </c>
@@ -1827,7 +1845,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="35" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>162</v>
       </c>
@@ -1838,7 +1856,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="36" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>170</v>
       </c>
@@ -1849,7 +1867,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>171</v>
       </c>
@@ -1857,7 +1875,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="38" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>172</v>
       </c>
@@ -1865,7 +1883,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="39" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>173</v>
       </c>
@@ -1873,7 +1891,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="40" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>174</v>
       </c>
@@ -1881,7 +1899,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="41" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>175</v>
       </c>
@@ -1889,7 +1907,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="42" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>176</v>
       </c>
@@ -1897,7 +1915,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="43" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>177</v>
       </c>
@@ -1905,7 +1923,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="44" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>15</v>
       </c>
@@ -1913,7 +1931,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="45" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>178</v>
       </c>
@@ -1924,7 +1942,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="46" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>179</v>
       </c>
@@ -1947,13 +1965,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B47">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="MLC2061579003"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:B47"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="260" orientation="portrait" horizontalDpi="203" verticalDpi="203" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Se configura pack kit transmisión cadena dorada DID-original R3
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="190">
   <si>
     <t>Número Publicación</t>
   </si>
@@ -586,6 +586,18 @@
   </si>
   <si>
     <t>MLC4105697882</t>
+  </si>
+  <si>
+    <t>MLC4152875310</t>
+  </si>
+  <si>
+    <t>MLC3965099640</t>
+  </si>
+  <si>
+    <t>MLC3841900316</t>
+  </si>
+  <si>
+    <t>MLC1914359413</t>
   </si>
 </sst>
 </file>
@@ -1172,7 +1184,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C45"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.6640625" bestFit="1" customWidth="1"/>
@@ -1519,6 +1531,30 @@
       </c>
       <c r="B42" t="s">
         <v>171</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>186</v>
+      </c>
+      <c r="B43" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>186</v>
+      </c>
+      <c r="B44" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>186</v>
+      </c>
+      <c r="B45" t="s">
+        <v>189</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
se configura cápsulas pedido bodega
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="192">
   <si>
     <t>Número Publicación</t>
   </si>
@@ -598,6 +598,12 @@
   </si>
   <si>
     <t>MLC1914359413</t>
+  </si>
+  <si>
+    <t>MLC4152901046</t>
+  </si>
+  <si>
+    <t>MLC2928322094</t>
   </si>
 </sst>
 </file>
@@ -1184,7 +1190,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:C45"/>
+  <dimension ref="A1:C48"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.6640625" bestFit="1" customWidth="1"/>
@@ -1554,6 +1560,30 @@
         <v>186</v>
       </c>
       <c r="B45" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>190</v>
+      </c>
+      <c r="B46" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>190</v>
+      </c>
+      <c r="B47" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>190</v>
+      </c>
+      <c r="B48" t="s">
         <v>189</v>
       </c>
     </row>

</xml_diff>

<commit_message>
se configuran polines xmax connected x6
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="OMITIDOS" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="193">
   <si>
     <t>Número Publicación</t>
   </si>
@@ -604,6 +604,9 @@
   </si>
   <si>
     <t>MLC2928322094</t>
+  </si>
+  <si>
+    <t>MLC4229052730</t>
   </si>
 </sst>
 </file>
@@ -1605,7 +1608,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C47"/>
+  <dimension ref="A1:C48"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.44140625" bestFit="1" customWidth="1"/>
@@ -2028,6 +2031,17 @@
       </c>
       <c r="C47">
         <v>4</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>192</v>
+      </c>
+      <c r="B48">
+        <v>12</v>
+      </c>
+      <c r="C48">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>